<commit_message>
revised files before submission
</commit_message>
<xml_diff>
--- a/data/romance_fraud_time.xlsx
+++ b/data/romance_fraud_time.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\nask.man.ac.uk\home$\Documents\GitHub\netflix_romancefraud\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA12859D-5D45-420E-8904-D4B09489FA76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7B750CD4-EC95-4A54-A9C8-834069E6B859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{43EE68DE-B5F0-484F-A17E-A9E7DAF0E414}"/>
   </bookViews>
@@ -4661,7 +4661,7 @@
         <v>464</v>
       </c>
       <c r="E64">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F64">
         <v>0</v>
@@ -4720,7 +4720,7 @@
         <v>472</v>
       </c>
       <c r="E65">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F65">
         <v>0</v>
@@ -4779,7 +4779,7 @@
         <v>505</v>
       </c>
       <c r="E66">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F66">
         <v>0</v>
@@ -4838,7 +4838,7 @@
         <v>517</v>
       </c>
       <c r="E67">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F67">
         <v>0</v>
@@ -4897,7 +4897,7 @@
         <v>454</v>
       </c>
       <c r="E68">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F68">
         <v>0</v>
@@ -4956,7 +4956,7 @@
         <v>508</v>
       </c>
       <c r="E69">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F69">
         <v>0</v>
@@ -5015,7 +5015,7 @@
         <v>499</v>
       </c>
       <c r="E70">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F70">
         <v>0</v>
@@ -5074,7 +5074,7 @@
         <v>447</v>
       </c>
       <c r="E71">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F71">
         <v>0</v>
@@ -5133,7 +5133,7 @@
         <v>469</v>
       </c>
       <c r="E72">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F72">
         <v>0</v>
@@ -5192,7 +5192,7 @@
         <v>465</v>
       </c>
       <c r="E73">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F73">
         <v>0</v>
@@ -5251,7 +5251,7 @@
         <v>444</v>
       </c>
       <c r="E74">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F74">
         <v>0</v>
@@ -5310,7 +5310,7 @@
         <v>432</v>
       </c>
       <c r="E75">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F75">
         <v>0</v>
@@ -5369,7 +5369,7 @@
         <v>518</v>
       </c>
       <c r="E76">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F76">
         <v>0</v>
@@ -5428,7 +5428,7 @@
         <v>616</v>
       </c>
       <c r="E77">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F77">
         <v>0</v>
@@ -5487,7 +5487,7 @@
         <v>640</v>
       </c>
       <c r="E78">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F78">
         <v>0</v>
@@ -5546,7 +5546,7 @@
         <v>605</v>
       </c>
       <c r="E79">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F79">
         <v>1</v>
@@ -5605,7 +5605,7 @@
         <v>623</v>
       </c>
       <c r="E80">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F80">
         <v>1</v>
@@ -5664,7 +5664,7 @@
         <v>705</v>
       </c>
       <c r="E81">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F81">
         <v>1</v>
@@ -5723,7 +5723,7 @@
         <v>626</v>
       </c>
       <c r="E82">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F82">
         <v>1</v>
@@ -5782,10 +5782,10 @@
         <v>615</v>
       </c>
       <c r="E83">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F83">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G83">
         <v>0</v>
@@ -5841,10 +5841,10 @@
         <v>654</v>
       </c>
       <c r="E84">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F84">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G84">
         <v>0</v>
@@ -5900,10 +5900,10 @@
         <v>736</v>
       </c>
       <c r="E85">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F85">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G85">
         <v>0</v>
@@ -5959,10 +5959,10 @@
         <v>901</v>
       </c>
       <c r="E86">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F86">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G86">
         <v>0</v>
@@ -6018,10 +6018,10 @@
         <v>710</v>
       </c>
       <c r="E87">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F87">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G87">
         <v>0</v>
@@ -6077,10 +6077,10 @@
         <v>802</v>
       </c>
       <c r="E88">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F88">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G88">
         <v>0</v>
@@ -6136,10 +6136,10 @@
         <v>758</v>
       </c>
       <c r="E89">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F89">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G89">
         <v>0</v>
@@ -6195,10 +6195,10 @@
         <v>781</v>
       </c>
       <c r="E90">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F90">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G90">
         <v>0</v>
@@ -6254,10 +6254,10 @@
         <v>785</v>
       </c>
       <c r="E91">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F91">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G91">
         <v>0</v>
@@ -6313,10 +6313,10 @@
         <v>680</v>
       </c>
       <c r="E92">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F92">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G92">
         <v>0</v>
@@ -6372,10 +6372,10 @@
         <v>781</v>
       </c>
       <c r="E93">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F93">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G93">
         <v>0</v>
@@ -6431,10 +6431,10 @@
         <v>741</v>
       </c>
       <c r="E94">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F94">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G94">
         <v>0</v>
@@ -6490,10 +6490,10 @@
         <v>660</v>
       </c>
       <c r="E95">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F95">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G95">
         <v>1</v>
@@ -6549,10 +6549,10 @@
         <v>684</v>
       </c>
       <c r="E96">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F96">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G96">
         <v>1</v>
@@ -6608,10 +6608,10 @@
         <v>671</v>
       </c>
       <c r="E97">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F97">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G97">
         <v>1</v>
@@ -6667,10 +6667,10 @@
         <v>583</v>
       </c>
       <c r="E98">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F98">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G98">
         <v>1</v>
@@ -6726,13 +6726,13 @@
         <v>671</v>
       </c>
       <c r="E99">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F99">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G99">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H99">
         <v>1</v>
@@ -6785,16 +6785,16 @@
         <v>767</v>
       </c>
       <c r="E100">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F100">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G100">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H100">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I100">
         <v>1</v>
@@ -6844,19 +6844,19 @@
         <v>668</v>
       </c>
       <c r="E101">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F101">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G101">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H101">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I101">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J101">
         <v>35</v>
@@ -6903,19 +6903,19 @@
         <v>656</v>
       </c>
       <c r="E102">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F102">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G102">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H102">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I102">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J102">
         <v>27</v>
@@ -6962,19 +6962,19 @@
         <v>662</v>
       </c>
       <c r="E103">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F103">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G103">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H103">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I103">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J103">
         <v>24</v>
@@ -7021,19 +7021,19 @@
         <v>662</v>
       </c>
       <c r="E104">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F104">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G104">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H104">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I104">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J104">
         <v>25</v>
@@ -7080,19 +7080,19 @@
         <v>662</v>
       </c>
       <c r="E105">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F105">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G105">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H105">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I105">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J105">
         <v>21</v>
@@ -7139,19 +7139,19 @@
         <v>636</v>
       </c>
       <c r="E106">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F106">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G106">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H106">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I106">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J106">
         <v>23</v>
@@ -7198,19 +7198,19 @@
         <v>616</v>
       </c>
       <c r="E107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J107">
         <v>32</v>
@@ -7257,19 +7257,19 @@
         <v>686</v>
       </c>
       <c r="E108">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F108">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G108">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H108">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I108">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J108">
         <v>37</v>
@@ -7316,19 +7316,19 @@
         <v>594</v>
       </c>
       <c r="E109">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F109">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G109">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H109">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I109">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J109">
         <v>47</v>
@@ -7375,19 +7375,19 @@
         <v>774</v>
       </c>
       <c r="E110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J110">
         <v>34</v>
@@ -7434,19 +7434,19 @@
         <v>642</v>
       </c>
       <c r="E111">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F111">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G111">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H111">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I111">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J111">
         <v>24</v>
@@ -7493,19 +7493,19 @@
         <v>657</v>
       </c>
       <c r="E112">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F112">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G112">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H112">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I112">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J112">
         <v>30</v>
@@ -7552,19 +7552,19 @@
         <v>756</v>
       </c>
       <c r="E113">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F113">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G113">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H113">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I113">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J113">
         <v>30</v>
@@ -7611,19 +7611,19 @@
         <v>830</v>
       </c>
       <c r="E114">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F114">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G114">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H114">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I114">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J114">
         <v>27</v>
@@ -7670,19 +7670,19 @@
         <v>867</v>
       </c>
       <c r="E115">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F115">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G115">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H115">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I115">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J115">
         <v>31</v>
@@ -7729,19 +7729,19 @@
         <v>686</v>
       </c>
       <c r="E116">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F116">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G116">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H116">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I116">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J116">
         <v>53</v>
@@ -7788,19 +7788,19 @@
         <v>759</v>
       </c>
       <c r="E117">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F117">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G117">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H117">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I117">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J117">
         <v>35</v>
@@ -7847,19 +7847,19 @@
         <v>695</v>
       </c>
       <c r="E118">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F118">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G118">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H118">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I118">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J118">
         <v>39</v>
@@ -7906,19 +7906,19 @@
         <v>662</v>
       </c>
       <c r="E119">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F119">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G119">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H119">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I119">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J119">
         <v>36</v>

</xml_diff>